<commit_message>
fix: preserve CSV boundaries and formula quoting
</commit_message>
<xml_diff>
--- a/src/__fixtures__/xlsx/basic-types.xlsx
+++ b/src/__fixtures__/xlsx/basic-types.xlsx
@@ -32,16 +32,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
   <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -185,7 +181,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -271,7 +267,6 @@
       <c r="D6" t="b">
         <v>1</v>
       </c>
-      <c r="E6" t="str"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
fix: preserve CSV boundaries and formula quoting (#126)
* fix: preserve CSV boundaries and formula quoting

* fix: quote overlapping CSV separators
</commit_message>
<xml_diff>
--- a/src/__fixtures__/xlsx/basic-types.xlsx
+++ b/src/__fixtures__/xlsx/basic-types.xlsx
@@ -32,16 +32,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
   <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -185,7 +181,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -271,7 +267,6 @@
       <c r="D6" t="b">
         <v>1</v>
       </c>
-      <c r="E6" t="str"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>